<commit_message>
Enhance apartment management system with rental features and ownership transitions
- Increased service timeout duration in OfficeObjectManager for better handling of long operations.
- Updated PlayerSuccessTracker to count rented apartments alongside owned ones.
- Introduced new apartment rental functionality in PropertyManager, allowing players to rent apartments with appropriate state management.
- Implemented methods for canceling apartment rentals and selling apartments, ensuring proper state transitions and financial adjustments.
- Added tests for apartment rental and ownership scenarios, ensuring correct behavior for purchasing, renting, and canceling apartments.
- Enhanced persistence logic to correctly save and load apartment rental states.
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99173302-A5DD-4B66-868E-CBCB9F459E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3549CD0A-5FE7-4F94-8D6D-0008B32FBF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="175">
   <si>
     <t>Context</t>
   </si>
@@ -531,6 +531,36 @@
   </si>
   <si>
     <t>Change cement props coordinates/heading</t>
+  </si>
+  <si>
+    <t>TO CHECK</t>
+  </si>
+  <si>
+    <t>Bricks</t>
+  </si>
+  <si>
+    <t>Bricks props not on flatbed + add more bricks</t>
+  </si>
+  <si>
+    <t>Despawn</t>
+  </si>
+  <si>
+    <t>Persistence</t>
+  </si>
+  <si>
+    <t>Notified an issue where the Hired NPC is not saved in the save even when saving the game</t>
+  </si>
+  <si>
+    <t>Extant the timeout delay</t>
+  </si>
+  <si>
+    <t>Notified a bug when purchasing a new apartment doesn't close the previous one</t>
+  </si>
+  <si>
+    <t>Delete entering/existed apartment notification</t>
+  </si>
+  <si>
+    <t>Add persistence to trucks, personal vehicles (color, modifications,…)</t>
   </si>
 </sst>
 </file>
@@ -596,30 +626,6 @@
   <dxfs count="6">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -648,6 +654,30 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -662,17 +692,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048576" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:F1048576" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F82">
-    <sortCondition ref="A1:A1048576"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048574" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:F1048574" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F88">
+    <sortCondition ref="A1:A1048574"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D467D48C-0EF7-43DB-9548-E040B8C5E91C}" name="Context"/>
     <tableColumn id="2" xr3:uid="{C2789722-93FA-4F2B-B083-D7D35A464CD9}" name="SubContext"/>
     <tableColumn id="3" xr3:uid="{94D8CD95-F067-44E9-9E87-1E09A248172F}" name="MenuPath"/>
-    <tableColumn id="4" xr3:uid="{F9C9C160-AA0D-435D-B307-ADA3AE42D618}" name="Type" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{0D23576C-5BB9-4211-9146-D3B59BC83479}" name="Status" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{F9C9C160-AA0D-435D-B307-ADA3AE42D618}" name="Type" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{0D23576C-5BB9-4211-9146-D3B59BC83479}" name="Status" dataDxfId="4"/>
     <tableColumn id="6" xr3:uid="{3AB2878E-83B0-4A29-8281-2817F20C1279}" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -996,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C35E873C-977B-43F9-B6E9-42F137FEA842}">
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -1004,7 +1034,7 @@
     <col min="3" max="3" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.42578125" style="3" customWidth="1"/>
     <col min="5" max="5" width="12.7109375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="180.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="133.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1038,7 +1068,7 @@
         <v>97</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
         <v>108</v>
@@ -1055,7 +1085,7 @@
         <v>71</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="F3" t="s">
         <v>110</v>
@@ -1072,7 +1102,7 @@
         <v>71</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="F4" t="s">
         <v>111</v>
@@ -1094,19 +1124,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>168</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1114,16 +1144,16 @@
         <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1131,16 +1161,16 @@
         <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1148,16 +1178,16 @@
         <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>123</v>
+        <v>63</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F9" t="s">
-        <v>124</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1174,84 +1204,75 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>123</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F12" t="s">
-        <v>16</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F13" t="s">
-        <v>17</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" t="s">
-        <v>19</v>
+        <v>73</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F14" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1271,7 +1292,7 @@
         <v>7</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1279,19 +1300,19 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F16" t="s">
-        <v>77</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1299,19 +1320,19 @@
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1319,19 +1340,19 @@
         <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>15</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F18" t="s">
-        <v>98</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1339,19 +1360,19 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F19" t="s">
-        <v>107</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1359,78 +1380,87 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>126</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>127</v>
+        <v>78</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F20" t="s">
-        <v>128</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>102</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="C21" t="s">
+        <v>96</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F21" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>95</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F22" t="s">
-        <v>34</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>126</v>
+      </c>
+      <c r="C23" t="s">
+        <v>127</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F23" t="s">
-        <v>39</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>69</v>
@@ -1439,7 +1469,7 @@
         <v>7</v>
       </c>
       <c r="F24" t="s">
-        <v>41</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1447,16 +1477,16 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F25" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1464,7 +1494,7 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>69</v>
@@ -1473,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="F26" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1481,7 +1511,7 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>69</v>
@@ -1490,7 +1520,7 @@
         <v>7</v>
       </c>
       <c r="F27" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1498,7 +1528,7 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>69</v>
@@ -1507,7 +1537,7 @@
         <v>7</v>
       </c>
       <c r="F28" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1515,16 +1545,16 @@
         <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F29" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1532,7 +1562,7 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>69</v>
@@ -1541,7 +1571,7 @@
         <v>7</v>
       </c>
       <c r="F30" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1549,16 +1579,16 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1566,16 +1596,16 @@
         <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F32" t="s">
-        <v>115</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1583,7 +1613,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>156</v>
+        <v>53</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>69</v>
@@ -1592,66 +1622,66 @@
         <v>7</v>
       </c>
       <c r="F33" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>129</v>
+        <v>7</v>
       </c>
       <c r="F35" t="s">
-        <v>23</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>24</v>
+        <v>156</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F36" t="s">
-        <v>20</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>70</v>
@@ -1660,7 +1690,7 @@
         <v>7</v>
       </c>
       <c r="F37" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1668,19 +1698,16 @@
         <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
-      </c>
-      <c r="C38" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F38" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1688,7 +1715,7 @@
         <v>21</v>
       </c>
       <c r="B39" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>70</v>
@@ -1697,7 +1724,7 @@
         <v>7</v>
       </c>
       <c r="F39" t="s">
-        <v>113</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1705,16 +1732,16 @@
         <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>109</v>
+        <v>25</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F40" t="s">
-        <v>116</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1722,16 +1749,19 @@
         <v>21</v>
       </c>
       <c r="B41" t="s">
-        <v>109</v>
+        <v>14</v>
+      </c>
+      <c r="C41" t="s">
+        <v>27</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F41" t="s">
-        <v>117</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1748,49 +1778,49 @@
         <v>7</v>
       </c>
       <c r="F42" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="B43" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="F43" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="B44" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>7</v>
+        <v>165</v>
       </c>
       <c r="F44" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="B45" t="s">
-        <v>138</v>
+        <v>6</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>70</v>
@@ -1799,24 +1829,24 @@
         <v>7</v>
       </c>
       <c r="F45" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="B46" t="s">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="F46" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1824,16 +1854,16 @@
         <v>131</v>
       </c>
       <c r="B47" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F47" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1841,24 +1871,24 @@
         <v>131</v>
       </c>
       <c r="B48" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F48" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="B49" t="s">
-        <v>6</v>
+        <v>138</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>70</v>
@@ -1867,15 +1897,15 @@
         <v>7</v>
       </c>
       <c r="F49" t="s">
-        <v>8</v>
+        <v>139</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="B50" t="s">
-        <v>6</v>
+        <v>140</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>70</v>
@@ -1884,67 +1914,58 @@
         <v>7</v>
       </c>
       <c r="F50" t="s">
-        <v>66</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="B51" t="s">
-        <v>55</v>
-      </c>
-      <c r="C51" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F51" t="s">
-        <v>82</v>
+        <v>142</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="B52" t="s">
-        <v>55</v>
-      </c>
-      <c r="C52" t="s">
-        <v>81</v>
+        <v>154</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F52" t="s">
-        <v>84</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
-      </c>
-      <c r="C53" t="s">
-        <v>81</v>
+        <v>163</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F53" t="s">
-        <v>90</v>
+        <v>164</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -1952,7 +1973,7 @@
         <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>85</v>
+        <v>6</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>70</v>
@@ -1961,7 +1982,7 @@
         <v>7</v>
       </c>
       <c r="F54" t="s">
-        <v>87</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -1969,7 +1990,7 @@
         <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>88</v>
+        <v>6</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>70</v>
@@ -1978,7 +1999,7 @@
         <v>7</v>
       </c>
       <c r="F55" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -1986,16 +2007,19 @@
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>91</v>
+        <v>55</v>
+      </c>
+      <c r="C56" t="s">
+        <v>81</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F56" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2009,13 +2033,13 @@
         <v>81</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F57" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2023,19 +2047,19 @@
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F58" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2043,75 +2067,81 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F59" t="s">
-        <v>143</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F60" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>36</v>
+        <v>91</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F61" t="s">
-        <v>37</v>
+        <v>92</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>36</v>
+        <v>55</v>
+      </c>
+      <c r="C62" t="s">
+        <v>81</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F62" t="s">
-        <v>130</v>
+        <v>83</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>134</v>
+        <v>99</v>
+      </c>
+      <c r="C63" t="s">
+        <v>100</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>70</v>
@@ -2120,32 +2150,32 @@
         <v>7</v>
       </c>
       <c r="F63" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B64" t="s">
-        <v>161</v>
+        <v>22</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F64" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>158</v>
+        <v>35</v>
       </c>
       <c r="B65" t="s">
-        <v>159</v>
+        <v>46</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>69</v>
@@ -2154,66 +2184,66 @@
         <v>7</v>
       </c>
       <c r="F65" t="s">
-        <v>160</v>
+        <v>47</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F66" t="s">
-        <v>151</v>
+        <v>37</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="B67" t="s">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F67" t="s">
-        <v>152</v>
+        <v>130</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>104</v>
+        <v>35</v>
       </c>
       <c r="B68" t="s">
-        <v>105</v>
+        <v>134</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F68" t="s">
-        <v>106</v>
+        <v>135</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="B69" t="s">
-        <v>10</v>
+        <v>161</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>69</v>
@@ -2222,15 +2252,15 @@
         <v>7</v>
       </c>
       <c r="F69" t="s">
-        <v>11</v>
+        <v>162</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>9</v>
+        <v>158</v>
       </c>
       <c r="B70" t="s">
-        <v>10</v>
+        <v>159</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>69</v>
@@ -2239,64 +2269,58 @@
         <v>7</v>
       </c>
       <c r="F70" t="s">
-        <v>12</v>
+        <v>160</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>9</v>
+        <v>149</v>
       </c>
       <c r="B71" t="s">
-        <v>63</v>
-      </c>
-      <c r="C71" t="s">
-        <v>64</v>
+        <v>150</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F71" t="s">
-        <v>62</v>
+        <v>151</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>9</v>
+        <v>149</v>
       </c>
       <c r="B72" t="s">
-        <v>63</v>
-      </c>
-      <c r="C72" t="s">
-        <v>64</v>
+        <v>150</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E72" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F72" t="s">
-        <v>65</v>
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>9</v>
+        <v>104</v>
       </c>
       <c r="B73" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F73" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2304,19 +2328,16 @@
         <v>9</v>
       </c>
       <c r="B74" t="s">
-        <v>6</v>
-      </c>
-      <c r="C74" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F74" t="s">
-        <v>112</v>
+        <v>11</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2324,19 +2345,16 @@
         <v>9</v>
       </c>
       <c r="B75" t="s">
-        <v>6</v>
-      </c>
-      <c r="C75" t="s">
-        <v>114</v>
+        <v>10</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F75" t="s">
-        <v>112</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2344,7 +2362,10 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>114</v>
+        <v>63</v>
+      </c>
+      <c r="C76" t="s">
+        <v>64</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>70</v>
@@ -2353,7 +2374,7 @@
         <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>119</v>
+        <v>62</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2361,16 +2382,19 @@
         <v>9</v>
       </c>
       <c r="B77" t="s">
-        <v>114</v>
+        <v>63</v>
+      </c>
+      <c r="C77" t="s">
+        <v>64</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F77" t="s">
-        <v>120</v>
+        <v>65</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2378,16 +2402,16 @@
         <v>9</v>
       </c>
       <c r="B78" t="s">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F78" t="s">
-        <v>121</v>
+        <v>86</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2395,7 +2419,10 @@
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>114</v>
+        <v>6</v>
+      </c>
+      <c r="C79" t="s">
+        <v>61</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>70</v>
@@ -2404,7 +2431,7 @@
         <v>7</v>
       </c>
       <c r="F79" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -2412,7 +2439,10 @@
         <v>9</v>
       </c>
       <c r="B80" t="s">
-        <v>144</v>
+        <v>6</v>
+      </c>
+      <c r="C80" t="s">
+        <v>114</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>70</v>
@@ -2421,7 +2451,7 @@
         <v>7</v>
       </c>
       <c r="F80" t="s">
-        <v>145</v>
+        <v>112</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2429,16 +2459,16 @@
         <v>9</v>
       </c>
       <c r="B81" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F81" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -2446,7 +2476,7 @@
         <v>9</v>
       </c>
       <c r="B82" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>69</v>
@@ -2455,42 +2485,145 @@
         <v>7</v>
       </c>
       <c r="F82" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>131</v>
+        <v>9</v>
       </c>
       <c r="B83" t="s">
-        <v>163</v>
+        <v>114</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F83" t="s">
-        <v>164</v>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>9</v>
+      </c>
+      <c r="B84" t="s">
+        <v>114</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F84" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>9</v>
+      </c>
+      <c r="B85" t="s">
+        <v>144</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F85" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>9</v>
+      </c>
+      <c r="B86" t="s">
+        <v>144</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F86" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>9</v>
+      </c>
+      <c r="B87" t="s">
+        <v>144</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F87" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>9</v>
+      </c>
+      <c r="B88" t="s">
+        <v>166</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F88" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>9</v>
+      </c>
+      <c r="B89" t="s">
+        <v>169</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F89" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="E1:E73 F3:F12 F14:F35 F37:F73 E74:F74 F75:F80 E75:E1048576">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+  <conditionalFormatting sqref="F3:F34 F36:F72 E73:F73 F74:F79 E74:E1048576 E1:E72">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"TO CHECK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"NOK"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Implement finance snapshot clearing in persistence management and add corresponding unit test
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F81FD7-820F-4A9C-AFE5-F7CF193C8382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C84737-E877-4A62-85E3-6951414B0B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="176">
   <si>
     <t>Context</t>
   </si>
@@ -558,9 +558,6 @@
   </si>
   <si>
     <t>Market</t>
-  </si>
-  <si>
-    <t>Delete everything about the market</t>
   </si>
   <si>
     <t>Add a supply and demand mechanism</t>
@@ -713,18 +710,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048573" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:F1048573" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048572" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:F1048572" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}">
     <filterColumn colId="3">
       <filters blank="1">
         <filter val="Bug"/>
-        <filter val="Change"/>
         <filter val="Delete"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048573">
-    <sortCondition ref="A1:A1048573"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048572">
+    <sortCondition ref="A1:A1048572"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D467D48C-0EF7-43DB-9548-E040B8C5E91C}" name="Context"/>
@@ -1055,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C35E873C-977B-43F9-B6E9-42F137FEA842}">
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -1168,7 +1164,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>56</v>
       </c>
@@ -1270,7 +1266,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>56</v>
       </c>
@@ -1287,7 +1283,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>71</v>
       </c>
@@ -1304,7 +1300,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1344,7 +1340,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1378,13 +1374,13 @@
         <v>70</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F18" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1464,55 +1460,55 @@
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="B23" t="s">
-        <v>173</v>
+        <v>92</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F23" t="s">
-        <v>174</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F24" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F25" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1520,7 +1516,7 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>68</v>
@@ -1529,7 +1525,7 @@
         <v>7</v>
       </c>
       <c r="F26" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1537,7 +1533,7 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>68</v>
@@ -1546,7 +1542,7 @@
         <v>7</v>
       </c>
       <c r="F27" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1554,7 +1550,7 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>68</v>
@@ -1563,7 +1559,7 @@
         <v>7</v>
       </c>
       <c r="F28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1571,7 +1567,7 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>68</v>
@@ -1580,7 +1576,7 @@
         <v>7</v>
       </c>
       <c r="F29" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1597,7 +1593,7 @@
         <v>7</v>
       </c>
       <c r="F30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1605,50 +1601,50 @@
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F31" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F32" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F33" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1656,7 +1652,7 @@
         <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>95</v>
@@ -1665,24 +1661,24 @@
         <v>7</v>
       </c>
       <c r="F34" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>31</v>
       </c>
       <c r="B35" t="s">
-        <v>29</v>
+        <v>154</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F35" t="s">
-        <v>113</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1690,7 +1686,7 @@
         <v>31</v>
       </c>
       <c r="B36" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>68</v>
@@ -1699,41 +1695,41 @@
         <v>7</v>
       </c>
       <c r="F36" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B37" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F37" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F38" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1741,24 +1737,24 @@
         <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="F39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>69</v>
@@ -1767,15 +1763,18 @@
         <v>7</v>
       </c>
       <c r="F40" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>24</v>
+        <v>14</v>
+      </c>
+      <c r="C41" t="s">
+        <v>26</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>69</v>
@@ -1784,18 +1783,15 @@
         <v>7</v>
       </c>
       <c r="F41" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
-      </c>
-      <c r="C42" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>69</v>
@@ -1804,7 +1800,7 @@
         <v>7</v>
       </c>
       <c r="F42" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1812,16 +1808,16 @@
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>7</v>
+        <v>163</v>
       </c>
       <c r="F43" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1838,24 +1834,24 @@
         <v>163</v>
       </c>
       <c r="F44" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>163</v>
+        <v>7</v>
       </c>
       <c r="F45" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1863,41 +1859,41 @@
         <v>20</v>
       </c>
       <c r="B46" t="s">
-        <v>6</v>
+        <v>167</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F46" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B47" t="s">
-        <v>167</v>
+        <v>130</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="F47" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>129</v>
       </c>
       <c r="B48" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>69</v>
@@ -1906,15 +1902,15 @@
         <v>7</v>
       </c>
       <c r="F48" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>129</v>
       </c>
       <c r="B49" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>69</v>
@@ -1923,15 +1919,15 @@
         <v>7</v>
       </c>
       <c r="F49" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>129</v>
       </c>
       <c r="B50" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>69</v>
@@ -1940,66 +1936,66 @@
         <v>7</v>
       </c>
       <c r="F50" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>129</v>
       </c>
       <c r="B51" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F51" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>129</v>
       </c>
       <c r="B52" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F52" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>129</v>
       </c>
       <c r="B53" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F53" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>69</v>
@@ -2008,10 +2004,10 @@
         <v>7</v>
       </c>
       <c r="F54" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -2025,15 +2021,18 @@
         <v>7</v>
       </c>
       <c r="F55" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>6</v>
+        <v>54</v>
+      </c>
+      <c r="C56" t="s">
+        <v>79</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>69</v>
@@ -2042,10 +2041,10 @@
         <v>7</v>
       </c>
       <c r="F56" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>3</v>
       </c>
@@ -2062,27 +2061,27 @@
         <v>7</v>
       </c>
       <c r="F57" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="C58" t="s">
         <v>79</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F58" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2090,27 +2089,24 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>89</v>
-      </c>
-      <c r="C59" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F59" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>69</v>
@@ -2119,61 +2115,64 @@
         <v>7</v>
       </c>
       <c r="F60" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F61" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>89</v>
+        <v>54</v>
+      </c>
+      <c r="C62" t="s">
+        <v>79</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F62" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>54</v>
+        <v>97</v>
       </c>
       <c r="C63" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F63" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2181,36 +2180,33 @@
         <v>3</v>
       </c>
       <c r="B64" t="s">
-        <v>97</v>
-      </c>
-      <c r="C64" t="s">
-        <v>98</v>
+        <v>21</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F64" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="B65" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F65" t="s">
-        <v>141</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2218,19 +2214,19 @@
         <v>34</v>
       </c>
       <c r="B66" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F66" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>34</v>
       </c>
@@ -2244,15 +2240,15 @@
         <v>7</v>
       </c>
       <c r="F67" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>34</v>
       </c>
       <c r="B68" t="s">
-        <v>35</v>
+        <v>132</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>69</v>
@@ -2261,32 +2257,32 @@
         <v>7</v>
       </c>
       <c r="F68" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>34</v>
       </c>
       <c r="B69" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F69" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
     </row>
     <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>34</v>
+        <v>156</v>
       </c>
       <c r="B70" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>68</v>
@@ -2295,15 +2291,15 @@
         <v>7</v>
       </c>
       <c r="F70" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="B71" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>68</v>
@@ -2312,7 +2308,7 @@
         <v>7</v>
       </c>
       <c r="F71" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
     </row>
     <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2329,41 +2325,41 @@
         <v>7</v>
       </c>
       <c r="F72" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>147</v>
+        <v>102</v>
       </c>
       <c r="B73" t="s">
-        <v>148</v>
+        <v>103</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F73" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>102</v>
+        <v>9</v>
       </c>
       <c r="B74" t="s">
-        <v>103</v>
+        <v>10</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F74" t="s">
-        <v>104</v>
+        <v>11</v>
       </c>
     </row>
     <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2380,7 +2376,7 @@
         <v>7</v>
       </c>
       <c r="F75" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2388,19 +2384,22 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
+        <v>62</v>
+      </c>
+      <c r="C76" t="s">
+        <v>63</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>9</v>
       </c>
@@ -2417,18 +2416,15 @@
         <v>7</v>
       </c>
       <c r="F77" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>9</v>
       </c>
       <c r="B78" t="s">
-        <v>62</v>
-      </c>
-      <c r="C78" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>69</v>
@@ -2437,15 +2433,18 @@
         <v>7</v>
       </c>
       <c r="F78" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>83</v>
+        <v>6</v>
+      </c>
+      <c r="C79" t="s">
+        <v>60</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>69</v>
@@ -2454,10 +2453,10 @@
         <v>7</v>
       </c>
       <c r="F79" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>9</v>
       </c>
@@ -2465,7 +2464,7 @@
         <v>6</v>
       </c>
       <c r="C80" t="s">
-        <v>60</v>
+        <v>112</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>69</v>
@@ -2477,14 +2476,11 @@
         <v>110</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>9</v>
       </c>
       <c r="B81" t="s">
-        <v>6</v>
-      </c>
-      <c r="C81" t="s">
         <v>112</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -2494,10 +2490,10 @@
         <v>7</v>
       </c>
       <c r="F81" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>9</v>
       </c>
@@ -2505,13 +2501,13 @@
         <v>112</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F82" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2528,7 +2524,7 @@
         <v>7</v>
       </c>
       <c r="F83" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2539,21 +2535,21 @@
         <v>112</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F84" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>9</v>
       </c>
       <c r="B85" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>69</v>
@@ -2562,7 +2558,7 @@
         <v>7</v>
       </c>
       <c r="F85" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -2573,16 +2569,16 @@
         <v>142</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F86" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>9</v>
       </c>
@@ -2590,69 +2586,52 @@
         <v>142</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F87" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>9</v>
       </c>
       <c r="B88" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F88" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>9</v>
       </c>
       <c r="B89" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F89" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>9</v>
-      </c>
-      <c r="B90" t="s">
-        <v>167</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E90" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F90" t="s">
         <v>172</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="F35:F71 E72:F72 F73:F78 E73:E1048576 F3:F33 E1:E71">
+  <conditionalFormatting sqref="F34:F70 E71:F71 F72:F77 E72:E1048576 F3:F32 E1:E70">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"TO CHECK"</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: Introduce AmbientWorldDispatchText class for status normalization and job type formatting, and add corresponding unit tests
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C84737-E877-4A62-85E3-6951414B0B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49203622-1EA7-4065-90C8-7E94F015ED68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="177">
   <si>
     <t>Context</t>
   </si>
@@ -564,6 +564,9 @@
   </si>
   <si>
     <t>When starting a new save, the budget from the previsou save are taking into account in the next save. I guess the state.ini file in the scripts folder in the entry point for a new save. --&gt; Delete .state.ini file</t>
+  </si>
+  <si>
+    <t>Modify market to "supply an demand" mechanism</t>
   </si>
 </sst>
 </file>
@@ -719,7 +722,7 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048572">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F90">
     <sortCondition ref="A1:A1048572"/>
   </sortState>
   <tableColumns count="6">
@@ -1051,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C35E873C-977B-43F9-B6E9-42F137FEA842}">
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -1414,7 +1417,7 @@
         <v>95</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>7</v>
+        <v>163</v>
       </c>
       <c r="F20" t="s">
         <v>96</v>
@@ -1700,10 +1703,10 @@
     </row>
     <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B37" t="s">
-        <v>29</v>
+        <v>173</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>69</v>
@@ -1712,24 +1715,24 @@
         <v>7</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B38" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="F38" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1737,16 +1740,16 @@
         <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F39" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1754,7 +1757,7 @@
         <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>69</v>
@@ -1763,7 +1766,7 @@
         <v>7</v>
       </c>
       <c r="F40" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1771,10 +1774,7 @@
         <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
-      </c>
-      <c r="C41" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>69</v>
@@ -1783,7 +1783,7 @@
         <v>7</v>
       </c>
       <c r="F41" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1791,7 +1791,10 @@
         <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>6</v>
+        <v>14</v>
+      </c>
+      <c r="C42" t="s">
+        <v>26</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>69</v>
@@ -1800,24 +1803,24 @@
         <v>7</v>
       </c>
       <c r="F42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>163</v>
+        <v>7</v>
       </c>
       <c r="F43" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1834,58 +1837,58 @@
         <v>163</v>
       </c>
       <c r="F44" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>7</v>
+        <v>163</v>
       </c>
       <c r="F45" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>20</v>
       </c>
       <c r="B46" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F46" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" t="s">
         <v>167</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D47" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E47" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F47" t="s">
         <v>168</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>129</v>
-      </c>
-      <c r="B47" t="s">
-        <v>130</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F47" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1893,7 +1896,7 @@
         <v>129</v>
       </c>
       <c r="B48" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>69</v>
@@ -1902,7 +1905,7 @@
         <v>7</v>
       </c>
       <c r="F48" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1910,7 +1913,7 @@
         <v>129</v>
       </c>
       <c r="B49" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>69</v>
@@ -1919,7 +1922,7 @@
         <v>7</v>
       </c>
       <c r="F49" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1927,7 +1930,7 @@
         <v>129</v>
       </c>
       <c r="B50" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>69</v>
@@ -1936,7 +1939,7 @@
         <v>7</v>
       </c>
       <c r="F50" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1944,58 +1947,58 @@
         <v>129</v>
       </c>
       <c r="B51" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F51" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>129</v>
       </c>
       <c r="B52" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F52" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>129</v>
       </c>
       <c r="B53" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F53" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>3</v>
+        <v>129</v>
       </c>
       <c r="B54" t="s">
-        <v>6</v>
+        <v>161</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>69</v>
@@ -2004,7 +2007,7 @@
         <v>7</v>
       </c>
       <c r="F54" t="s">
-        <v>8</v>
+        <v>162</v>
       </c>
     </row>
     <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2021,7 +2024,7 @@
         <v>7</v>
       </c>
       <c r="F55" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2029,10 +2032,7 @@
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>54</v>
-      </c>
-      <c r="C56" t="s">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>69</v>
@@ -2041,7 +2041,7 @@
         <v>7</v>
       </c>
       <c r="F56" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
     </row>
     <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2061,7 +2061,7 @@
         <v>7</v>
       </c>
       <c r="F57" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2069,19 +2069,19 @@
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="C58" t="s">
         <v>79</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F58" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2089,16 +2089,19 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>83</v>
+        <v>89</v>
+      </c>
+      <c r="C59" t="s">
+        <v>79</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F59" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2106,7 +2109,7 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>69</v>
@@ -2115,7 +2118,7 @@
         <v>7</v>
       </c>
       <c r="F60" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2123,90 +2126,90 @@
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F61" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>54</v>
-      </c>
-      <c r="C62" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F62" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>97</v>
+        <v>54</v>
       </c>
       <c r="C63" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F63" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>3</v>
       </c>
       <c r="B64" t="s">
+        <v>97</v>
+      </c>
+      <c r="C64" t="s">
+        <v>98</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F64" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
         <v>21</v>
       </c>
-      <c r="D64" s="3" t="s">
+      <c r="D65" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E64" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="E65" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F65" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>34</v>
-      </c>
-      <c r="B65" t="s">
-        <v>45</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F65" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2214,16 +2217,16 @@
         <v>34</v>
       </c>
       <c r="B66" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F66" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2240,7 +2243,7 @@
         <v>7</v>
       </c>
       <c r="F67" t="s">
-        <v>128</v>
+        <v>36</v>
       </c>
     </row>
     <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2248,7 +2251,7 @@
         <v>34</v>
       </c>
       <c r="B68" t="s">
-        <v>132</v>
+        <v>35</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>69</v>
@@ -2257,7 +2260,7 @@
         <v>7</v>
       </c>
       <c r="F68" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2265,24 +2268,24 @@
         <v>34</v>
       </c>
       <c r="B69" t="s">
-        <v>159</v>
+        <v>132</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F69" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
     </row>
     <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>156</v>
+        <v>34</v>
       </c>
       <c r="B70" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>68</v>
@@ -2291,15 +2294,15 @@
         <v>7</v>
       </c>
       <c r="F70" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="B71" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>68</v>
@@ -2308,7 +2311,7 @@
         <v>7</v>
       </c>
       <c r="F71" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
     </row>
     <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2325,41 +2328,41 @@
         <v>7</v>
       </c>
       <c r="F72" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>147</v>
+      </c>
+      <c r="B73" t="s">
+        <v>148</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F73" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>102</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>103</v>
       </c>
-      <c r="D73" s="3" t="s">
+      <c r="D74" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E73" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F73" t="s">
+      <c r="E74" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F74" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>9</v>
-      </c>
-      <c r="B74" t="s">
-        <v>10</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E74" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F74" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2376,7 +2379,7 @@
         <v>7</v>
       </c>
       <c r="F75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2384,19 +2387,16 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>62</v>
-      </c>
-      <c r="C76" t="s">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2416,7 +2416,7 @@
         <v>7</v>
       </c>
       <c r="F77" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2424,7 +2424,10 @@
         <v>9</v>
       </c>
       <c r="B78" t="s">
-        <v>83</v>
+        <v>62</v>
+      </c>
+      <c r="C78" t="s">
+        <v>63</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>69</v>
@@ -2433,7 +2436,7 @@
         <v>7</v>
       </c>
       <c r="F78" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2441,10 +2444,7 @@
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>6</v>
-      </c>
-      <c r="C79" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>69</v>
@@ -2453,7 +2453,7 @@
         <v>7</v>
       </c>
       <c r="F79" t="s">
-        <v>110</v>
+        <v>84</v>
       </c>
     </row>
     <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2464,7 +2464,7 @@
         <v>6</v>
       </c>
       <c r="C80" t="s">
-        <v>112</v>
+        <v>60</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>69</v>
@@ -2481,6 +2481,9 @@
         <v>9</v>
       </c>
       <c r="B81" t="s">
+        <v>6</v>
+      </c>
+      <c r="C81" t="s">
         <v>112</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -2490,7 +2493,7 @@
         <v>7</v>
       </c>
       <c r="F81" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2501,13 +2504,13 @@
         <v>112</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F82" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2524,7 +2527,7 @@
         <v>7</v>
       </c>
       <c r="F83" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2535,13 +2538,13 @@
         <v>112</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F84" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2549,7 +2552,7 @@
         <v>9</v>
       </c>
       <c r="B85" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>69</v>
@@ -2558,10 +2561,10 @@
         <v>7</v>
       </c>
       <c r="F85" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>9</v>
       </c>
@@ -2569,16 +2572,16 @@
         <v>142</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F86" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>9</v>
       </c>
@@ -2586,46 +2589,63 @@
         <v>142</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F87" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>9</v>
       </c>
       <c r="B88" t="s">
-        <v>164</v>
+        <v>142</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F88" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>9</v>
       </c>
       <c r="B89" t="s">
+        <v>164</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F89" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>9</v>
+      </c>
+      <c r="B90" t="s">
         <v>167</v>
       </c>
-      <c r="D89" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E89" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F89" t="s">
+      <c r="D90" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F90" t="s">
         <v>172</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Refactor permit caption and location detail formatting, and add unit tests for new functionality
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49203622-1EA7-4065-90C8-7E94F015ED68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDAB4D7-578B-4CD7-943C-C467C9CE0B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -1417,7 +1417,7 @@
         <v>95</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="F20" t="s">
         <v>96</v>
@@ -1437,7 +1437,7 @@
         <v>95</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F21" t="s">
         <v>105</v>
@@ -1457,7 +1457,7 @@
         <v>95</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F22" t="s">
         <v>126</v>

</xml_diff>

<commit_message>
Refactor industry management and improve economic balance
- Introduced NonSinkDeliveryPayoutMultiplier to enhance delivery payouts for non-sink deliveries.
- Updated delivery profit calculation to use the new multiplier.
- Enhanced industry configuration to include emptying rates and owner cuts.
- Improved handling of boost inputs in industry recipes.
- Fixed issues with effective input/output capacity calculations.
- Adjusted fuel delivery price multiplier for better market alignment.
- Added comprehensive economy rebalance report outlining structural issues and proposed solutions.
- Updated commodity pricing and sink pressure metrics to improve gameplay balance.
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDAB4D7-578B-4CD7-943C-C467C9CE0B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C948D3-68AA-4A4D-8608-F2CC886096E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -461,9 +461,6 @@
     <t>Add plastic object coordinates</t>
   </si>
   <si>
-    <t>If vehicle outside garage, offic emenu option is "retreive" not "stored"</t>
-  </si>
-  <si>
     <t>Props cargo</t>
   </si>
   <si>
@@ -567,13 +564,16 @@
   </si>
   <si>
     <t>Modify market to "supply an demand" mechanism</t>
+  </si>
+  <si>
+    <t>Change moving object behaviour mechanism</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -602,8 +602,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -613,6 +620,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -625,11 +637,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -639,9 +652,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
@@ -713,8 +728,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048572" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:F1048572" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048571" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:F1048571" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}">
     <filterColumn colId="3">
       <filters blank="1">
         <filter val="Bug"/>
@@ -723,7 +738,7 @@
     </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F90">
-    <sortCondition ref="A1:A1048572"/>
+    <sortCondition ref="A1:A1048571"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D467D48C-0EF7-43DB-9548-E040B8C5E91C}" name="Context"/>
@@ -1113,7 +1128,7 @@
         <v>70</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F3" t="s">
         <v>108</v>
@@ -1130,7 +1145,7 @@
         <v>70</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F4" t="s">
         <v>109</v>
@@ -1147,7 +1162,7 @@
         <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1155,16 +1170,16 @@
         <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1266,7 +1281,7 @@
         <v>127</v>
       </c>
       <c r="F12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1283,7 +1298,7 @@
         <v>127</v>
       </c>
       <c r="F13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1380,7 +1395,7 @@
         <v>127</v>
       </c>
       <c r="F18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1644,7 +1659,7 @@
         <v>95</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F33" t="s">
         <v>55</v>
@@ -1663,7 +1678,7 @@
       <c r="E34" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="5" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1672,16 +1687,16 @@
         <v>31</v>
       </c>
       <c r="B35" t="s">
+        <v>153</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F35" t="s">
         <v>154</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F35" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1689,16 +1704,16 @@
         <v>31</v>
       </c>
       <c r="B36" t="s">
+        <v>172</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F36" t="s">
         <v>173</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F36" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1706,7 +1721,7 @@
         <v>31</v>
       </c>
       <c r="B37" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>69</v>
@@ -1715,7 +1730,7 @@
         <v>7</v>
       </c>
       <c r="F37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1834,7 +1849,7 @@
         <v>70</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F44" t="s">
         <v>114</v>
@@ -1851,7 +1866,7 @@
         <v>70</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F45" t="s">
         <v>115</v>
@@ -1879,7 +1894,7 @@
         <v>20</v>
       </c>
       <c r="B47" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>70</v>
@@ -1888,7 +1903,7 @@
         <v>127</v>
       </c>
       <c r="F47" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1964,7 +1979,7 @@
         <v>129</v>
       </c>
       <c r="B52" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>68</v>
@@ -1981,16 +1996,16 @@
         <v>129</v>
       </c>
       <c r="B53" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>7</v>
+        <v>162</v>
       </c>
       <c r="F53" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -1998,16 +2013,16 @@
         <v>129</v>
       </c>
       <c r="B54" t="s">
+        <v>160</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F54" t="s">
         <v>161</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F54" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2195,21 +2210,21 @@
         <v>99</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>3</v>
       </c>
       <c r="B65" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F65" t="s">
-        <v>141</v>
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2285,59 +2300,59 @@
         <v>34</v>
       </c>
       <c r="B70" t="s">
+        <v>158</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F70" t="s">
         <v>159</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F70" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>155</v>
+      </c>
+      <c r="B71" t="s">
         <v>156</v>
       </c>
-      <c r="B71" t="s">
+      <c r="D71" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F71" t="s">
         <v>157</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F71" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>146</v>
+      </c>
+      <c r="B72" t="s">
         <v>147</v>
       </c>
-      <c r="B72" t="s">
+      <c r="D72" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F72" t="s">
         <v>148</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F72" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>146</v>
+      </c>
+      <c r="B73" t="s">
         <v>147</v>
       </c>
-      <c r="B73" t="s">
-        <v>148</v>
-      </c>
       <c r="D73" s="3" t="s">
         <v>68</v>
       </c>
@@ -2345,7 +2360,7 @@
         <v>7</v>
       </c>
       <c r="F73" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2569,16 +2584,16 @@
         <v>9</v>
       </c>
       <c r="B86" t="s">
+        <v>141</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F86" t="s">
         <v>142</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E86" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F86" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -2586,7 +2601,7 @@
         <v>9</v>
       </c>
       <c r="B87" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>70</v>
@@ -2595,7 +2610,7 @@
         <v>7</v>
       </c>
       <c r="F87" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2603,7 +2618,7 @@
         <v>9</v>
       </c>
       <c r="B88" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>68</v>
@@ -2612,7 +2627,7 @@
         <v>7</v>
       </c>
       <c r="F88" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -2620,7 +2635,7 @@
         <v>9</v>
       </c>
       <c r="B89" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>70</v>
@@ -2629,7 +2644,7 @@
         <v>7</v>
       </c>
       <c r="F89" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2637,7 +2652,7 @@
         <v>9</v>
       </c>
       <c r="B90" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>68</v>
@@ -2646,12 +2661,12 @@
         <v>7</v>
       </c>
       <c r="F90" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="F34:F70 E71:F71 F72:F77 E72:E1048576 F3:F32 E1:E70">
+  <conditionalFormatting sqref="E70:F70 F71:F76 E71:E1048576 F3:F32 F34:F69 E1:E69">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"TO CHECK"</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: Enhance delivery progress tracking with NPC source and add unit tests for new functionality
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C948D3-68AA-4A4D-8608-F2CC886096E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B523BC6F-C2FD-4FEE-9BE2-FD51686617F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -2374,7 +2374,7 @@
         <v>70</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>7</v>
+        <v>162</v>
       </c>
       <c r="F74" t="s">
         <v>104</v>

</xml_diff>

<commit_message>
feat: Remove wood-related visual prop logic from FleetManager and update tests accordingly
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B523BC6F-C2FD-4FEE-9BE2-FD51686617F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F97FF1-FE0C-453A-94B1-0AA254009F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -734,6 +734,12 @@
       <filters blank="1">
         <filter val="Bug"/>
         <filter val="Delete"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters blank="1">
+        <filter val="NOK"/>
+        <filter val="TO CHECK"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1100,7 +1106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -1216,7 +1222,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -1267,7 +1273,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>56</v>
       </c>
@@ -1338,7 +1344,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1378,7 +1384,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1418,7 +1424,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -1438,7 +1444,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1458,7 +1464,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1648,7 +1654,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1889,7 +1895,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>20</v>
       </c>
@@ -2002,7 +2008,7 @@
         <v>70</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>162</v>
+        <v>7</v>
       </c>
       <c r="F53" t="s">
         <v>152</v>
@@ -2042,7 +2048,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>3</v>
       </c>
@@ -2050,10 +2056,10 @@
         <v>6</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>7</v>
+        <v>162</v>
       </c>
       <c r="F56" t="s">
         <v>65</v>
@@ -2596,7 +2602,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>9</v>
       </c>
@@ -2607,7 +2613,7 @@
         <v>70</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="F87" t="s">
         <v>144</v>

</xml_diff>

<commit_message>
feat: Implement global market persistence with loading and saving functionality, and add corresponding unit tests
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F97FF1-FE0C-453A-94B1-0AA254009F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA56CBA9-EA1C-4DC0-B16D-BB2866A56D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="173">
   <si>
     <t>Context</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Rocks props for tipper and brute trucks</t>
   </si>
   <si>
-    <t>Bricks props number should be increase on flatbed</t>
-  </si>
-  <si>
     <t>COMPANY HUB</t>
   </si>
   <si>
@@ -191,15 +188,9 @@
     <t xml:space="preserve">Owning </t>
   </si>
   <si>
-    <t>Owning mechanism to rework as the payer is given oney for industries it owns</t>
-  </si>
-  <si>
     <t>Franchise</t>
   </si>
   <si>
-    <t>Owning a store or a gas station should give player passive money each in-game week based on site frequency</t>
-  </si>
-  <si>
     <t>Notification</t>
   </si>
   <si>
@@ -230,9 +221,6 @@
     <t>Commercial Dealership &gt; Rent</t>
   </si>
   <si>
-    <t>Divide rent cost by 2</t>
-  </si>
-  <si>
     <t>Delete office garage blip</t>
   </si>
   <si>
@@ -428,24 +416,12 @@
     <t>INDUSTRY</t>
   </si>
   <si>
-    <t>Oil field</t>
-  </si>
-  <si>
-    <t>Increase Oil field capacity by x100</t>
-  </si>
-  <si>
     <t>Oil</t>
   </si>
   <si>
     <t>Change oil price</t>
   </si>
   <si>
-    <t>Refinery</t>
-  </si>
-  <si>
-    <t>Increase Refinery capacity by x100</t>
-  </si>
-  <si>
     <t>Productivity</t>
   </si>
   <si>
@@ -554,19 +530,31 @@
     <t>Add persistence to trucks, personal vehicles (color, modifications,…)</t>
   </si>
   <si>
-    <t>Market</t>
-  </si>
-  <si>
-    <t>Add a supply and demand mechanism</t>
-  </si>
-  <si>
     <t>When starting a new save, the budget from the previsou save are taking into account in the next save. I guess the state.ini file in the scripts folder in the entry point for a new save. --&gt; Delete .state.ini file</t>
   </si>
   <si>
-    <t>Modify market to "supply an demand" mechanism</t>
-  </si>
-  <si>
     <t>Change moving object behaviour mechanism</t>
+  </si>
+  <si>
+    <t>Contracts</t>
+  </si>
+  <si>
+    <t>Add contracts with supply and demand mechanism</t>
+  </si>
+  <si>
+    <t>Owning mechanism to rework as the payer is given money for industries it owns</t>
+  </si>
+  <si>
+    <t>Owning a store or a gas station should give player passive money each in-game week based on site frequency as while the site is filled with resources</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Reduce the upfront cost for hiring NPC</t>
+  </si>
+  <si>
+    <t>Rebalance renting cost</t>
   </si>
 </sst>
 </file>
@@ -728,23 +716,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048571" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:F1048571" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}">
-    <filterColumn colId="3">
-      <filters blank="1">
-        <filter val="Bug"/>
-        <filter val="Delete"/>
-      </filters>
-    </filterColumn>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048566" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:F1048566" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}">
     <filterColumn colId="4">
       <filters blank="1">
         <filter val="NOK"/>
-        <filter val="TO CHECK"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F90">
-    <sortCondition ref="A1:A1048571"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F89">
+    <sortCondition ref="A1:A1048566"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D467D48C-0EF7-43DB-9548-E040B8C5E91C}" name="Context"/>
@@ -1075,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C35E873C-977B-43F9-B6E9-42F137FEA842}">
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -1097,7 +1078,7 @@
         <v>5</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -1108,944 +1089,947 @@
     </row>
     <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="E2" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F6" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" t="s">
         <v>56</v>
-      </c>
-      <c r="B8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F8" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F9" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F12" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F13" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F14" t="s">
         <v>69</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
         <v>13</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" t="s">
         <v>14</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D17" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F17" t="s">
         <v>18</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F17" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" t="s">
         <v>74</v>
-      </c>
-      <c r="C18" t="s">
-        <v>75</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F18" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" t="s">
-        <v>77</v>
-      </c>
-      <c r="C19" t="s">
-        <v>76</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F19" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F20" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F21" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C22" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F22" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B23" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F23" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" t="s">
         <v>31</v>
       </c>
-      <c r="B24" t="s">
+      <c r="D24" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F24" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F25" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F25" t="s">
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="D26" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F26" t="s">
         <v>39</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F26" t="s">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="D27" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F27" t="s">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="D28" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" t="s">
         <v>43</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F28" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" t="s">
         <v>47</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F29" t="s">
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F30" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" t="s">
-        <v>47</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F30" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" t="s">
+      <c r="D31" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F31" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32" t="s">
-        <v>52</v>
-      </c>
       <c r="D32" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F32" t="s">
-        <v>53</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F33" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" t="s">
+        <v>145</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F35" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" t="s">
+        <v>166</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F36" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F37" t="s">
         <v>29</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" t="s">
-        <v>153</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F35" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" t="s">
-        <v>172</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F36" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" t="s">
-        <v>172</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F37" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F38" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B39" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="F39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B40" t="s">
         <v>23</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>20</v>
-      </c>
       <c r="B41" t="s">
-        <v>24</v>
+        <v>13</v>
+      </c>
+      <c r="C41" t="s">
+        <v>25</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F41" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
-      </c>
-      <c r="C42" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F42" t="s">
-        <v>27</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B43" t="s">
-        <v>6</v>
+        <v>103</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="F43" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" t="s">
+        <v>103</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F44" t="s">
         <v>111</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44" t="s">
-        <v>107</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="F44" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B45" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>162</v>
+        <v>7</v>
       </c>
       <c r="F45" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B46" t="s">
-        <v>6</v>
+        <v>158</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F46" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B47" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="F47" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>125</v>
+      </c>
+      <c r="B48" t="s">
+        <v>128</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F48" t="s">
         <v>129</v>
       </c>
-      <c r="B48" t="s">
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>125</v>
+      </c>
+      <c r="B49" t="s">
         <v>130</v>
       </c>
-      <c r="D48" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="D49" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F49" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>129</v>
-      </c>
-      <c r="B49" t="s">
-        <v>134</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F49" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B50" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F50" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B51" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F51" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B52" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F52" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="B53" t="s">
-        <v>151</v>
+        <v>6</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F53" t="s">
-        <v>152</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F54" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>6</v>
+        <v>51</v>
+      </c>
+      <c r="C55" t="s">
+        <v>75</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F55" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2053,127 +2037,130 @@
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>6</v>
+        <v>51</v>
+      </c>
+      <c r="C56" t="s">
+        <v>75</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>162</v>
+        <v>7</v>
       </c>
       <c r="F56" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>3</v>
       </c>
       <c r="B57" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="C57" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F57" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>54</v>
-      </c>
-      <c r="C58" t="s">
         <v>79</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F58" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>89</v>
-      </c>
-      <c r="C59" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F59" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F60" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>86</v>
+        <v>51</v>
+      </c>
+      <c r="C61" t="s">
+        <v>75</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F61" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>89</v>
+        <v>93</v>
+      </c>
+      <c r="C62" t="s">
+        <v>94</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F62" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2181,209 +2168,206 @@
         <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>54</v>
-      </c>
-      <c r="C63" t="s">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F63" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="B64" t="s">
-        <v>97</v>
-      </c>
-      <c r="C64" t="s">
-        <v>98</v>
+        <v>44</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F64" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="B65" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F65" t="s">
-        <v>176</v>
+        <v>35</v>
       </c>
     </row>
     <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>33</v>
+      </c>
+      <c r="B66" t="s">
         <v>34</v>
       </c>
-      <c r="B66" t="s">
-        <v>45</v>
-      </c>
       <c r="D66" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F66" t="s">
-        <v>46</v>
+        <v>124</v>
       </c>
     </row>
     <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B67" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F67" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B68" t="s">
-        <v>35</v>
+        <v>150</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F68" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>34</v>
+        <v>147</v>
       </c>
       <c r="B69" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F69" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>34</v>
+        <v>138</v>
       </c>
       <c r="B70" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F70" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="B71" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F71" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
     </row>
     <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>146</v>
+        <v>98</v>
       </c>
       <c r="B72" t="s">
-        <v>147</v>
+        <v>99</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="F72" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>146</v>
+        <v>9</v>
       </c>
       <c r="B73" t="s">
-        <v>147</v>
+        <v>10</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F73" t="s">
-        <v>149</v>
+        <v>11</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>102</v>
+        <v>9</v>
       </c>
       <c r="B74" t="s">
-        <v>103</v>
+        <v>59</v>
+      </c>
+      <c r="C74" t="s">
+        <v>60</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>162</v>
+        <v>7</v>
       </c>
       <c r="F74" t="s">
-        <v>104</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2391,164 +2375,161 @@
         <v>9</v>
       </c>
       <c r="B75" t="s">
-        <v>10</v>
+        <v>59</v>
+      </c>
+      <c r="C75" t="s">
+        <v>60</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F75" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>9</v>
       </c>
       <c r="B77" t="s">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="C77" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F77" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>9</v>
       </c>
       <c r="B78" t="s">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="C78" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F78" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F79" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>9</v>
       </c>
       <c r="B80" t="s">
-        <v>6</v>
-      </c>
-      <c r="C80" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E80" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F80" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>9</v>
       </c>
       <c r="B81" t="s">
-        <v>6</v>
-      </c>
-      <c r="C81" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F81" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>9</v>
       </c>
       <c r="B82" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F82" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>9</v>
       </c>
       <c r="B83" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F83" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -2556,123 +2537,72 @@
         <v>9</v>
       </c>
       <c r="B84" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F84" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>9</v>
       </c>
       <c r="B85" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F85" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>9</v>
       </c>
       <c r="B86" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F86" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>9</v>
       </c>
       <c r="B87" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="F87" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>9</v>
-      </c>
-      <c r="B88" t="s">
-        <v>141</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E88" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F88" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>9</v>
-      </c>
-      <c r="B89" t="s">
         <v>163</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E89" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F89" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>9</v>
-      </c>
-      <c r="B90" t="s">
-        <v>166</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E90" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F90" t="s">
-        <v>171</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="E70:F70 F71:F76 E71:E1048576 F3:F32 F34:F69 E1:E69">
+  <conditionalFormatting sqref="E66:F66 F67:F72 F3:F32 F34:F65 E1:E65 E67:E1048576">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"TO CHECK"</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: Implement CancelActiveRefuelDispatchForShutdown method and refactor shutdown logic
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB25D7C-BA74-462F-B753-4F2560DE1CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C18342-AD9B-4FA5-8EAA-1635730CF477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -730,7 +730,7 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}" name="Table1" displayName="Table1" ref="A1:F1048565" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:F1048565" xr:uid="{BB427F43-D77B-4D23-ABAD-8D570D743033}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F89">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F90">
     <sortCondition ref="A1:A1048565"/>
   </sortState>
   <tableColumns count="6">
@@ -1177,19 +1177,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>172</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="F7" t="s">
-        <v>54</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1197,16 +1197,16 @@
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1214,16 +1214,16 @@
         <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F9" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1231,16 +1231,16 @@
         <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>115</v>
+        <v>59</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F10" t="s">
-        <v>116</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1254,10 +1254,10 @@
         <v>64</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1265,16 +1265,16 @@
         <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>159</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1282,24 +1282,24 @@
         <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>65</v>
@@ -1308,27 +1308,24 @@
         <v>121</v>
       </c>
       <c r="F14" t="s">
-        <v>69</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>15</v>
+        <v>121</v>
+      </c>
+      <c r="F15" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1339,16 +1336,16 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="F16" t="s">
-        <v>16</v>
+        <v>7</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1359,16 +1356,16 @@
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F17" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1376,19 +1373,19 @@
         <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F18" t="s">
-        <v>162</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1396,19 +1393,19 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F19" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1416,19 +1413,19 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1448,7 +1445,7 @@
         <v>121</v>
       </c>
       <c r="F21" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1456,10 +1453,10 @@
         <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>90</v>
@@ -1468,41 +1465,44 @@
         <v>121</v>
       </c>
       <c r="F22" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>118</v>
+      </c>
+      <c r="C23" t="s">
+        <v>119</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F23" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>95</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>152</v>
+        <v>7</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1510,16 +1510,16 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>7</v>
+        <v>152</v>
       </c>
       <c r="F25" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1527,7 +1527,7 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>64</v>
@@ -1536,7 +1536,7 @@
         <v>7</v>
       </c>
       <c r="F26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1544,7 +1544,7 @@
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>64</v>
@@ -1553,7 +1553,7 @@
         <v>7</v>
       </c>
       <c r="F27" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1561,7 +1561,7 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>64</v>
@@ -1570,7 +1570,7 @@
         <v>7</v>
       </c>
       <c r="F28" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1578,7 +1578,7 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>64</v>
@@ -1587,7 +1587,7 @@
         <v>7</v>
       </c>
       <c r="F29" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1604,7 +1604,7 @@
         <v>7</v>
       </c>
       <c r="F30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1612,16 +1612,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F31" t="s">
-        <v>166</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1629,16 +1629,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>152</v>
+        <v>7</v>
       </c>
       <c r="F32" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1646,16 +1646,16 @@
         <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="F33" t="s">
-        <v>52</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1663,16 +1663,16 @@
         <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>90</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>107</v>
+        <v>121</v>
+      </c>
+      <c r="F34" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1680,16 +1680,16 @@
         <v>30</v>
       </c>
       <c r="B35" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F35" t="s">
-        <v>144</v>
+      <c r="F35" s="5" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1697,33 +1697,33 @@
         <v>30</v>
       </c>
       <c r="B36" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>64</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>152</v>
+        <v>7</v>
       </c>
       <c r="F36" t="s">
-        <v>165</v>
+        <v>144</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B37" t="s">
-        <v>28</v>
+        <v>164</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>7</v>
+        <v>152</v>
       </c>
       <c r="F37" t="s">
-        <v>29</v>
+        <v>165</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1731,16 +1731,16 @@
         <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>172</v>
+        <v>28</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F38" t="s">
-        <v>174</v>
+        <v>29</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1751,30 +1751,30 @@
         <v>172</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F39" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B40" t="s">
-        <v>20</v>
+        <v>172</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F40" t="s">
-        <v>21</v>
+        <v>175</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1782,16 +1782,16 @@
         <v>19</v>
       </c>
       <c r="B41" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>24</v>
+        <v>121</v>
+      </c>
+      <c r="F41" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1799,13 +1799,16 @@
         <v>19</v>
       </c>
       <c r="B42" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>7</v>
+        <v>152</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1813,16 +1816,13 @@
         <v>19</v>
       </c>
       <c r="B43" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F43" t="s">
-        <v>108</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1839,7 +1839,7 @@
         <v>152</v>
       </c>
       <c r="F44" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -1847,16 +1847,16 @@
         <v>19</v>
       </c>
       <c r="B45" t="s">
-        <v>6</v>
+        <v>102</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>152</v>
       </c>
       <c r="F45" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1864,19 +1864,16 @@
         <v>19</v>
       </c>
       <c r="B46" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="F46" t="s">
-        <v>26</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1884,16 +1881,19 @@
         <v>19</v>
       </c>
       <c r="B47" t="s">
-        <v>168</v>
+        <v>13</v>
+      </c>
+      <c r="C47" t="s">
+        <v>25</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="F47" t="s">
-        <v>169</v>
+        <v>26</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1901,33 +1901,33 @@
         <v>19</v>
       </c>
       <c r="B48" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="F48" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>123</v>
+        <v>19</v>
       </c>
       <c r="B49" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F49" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -1935,16 +1935,16 @@
         <v>123</v>
       </c>
       <c r="B50" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F50" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -1952,16 +1952,16 @@
         <v>123</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F51" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -1969,16 +1969,16 @@
         <v>123</v>
       </c>
       <c r="B52" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F52" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -1986,33 +1986,33 @@
         <v>123</v>
       </c>
       <c r="B53" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F53" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>3</v>
+        <v>123</v>
       </c>
       <c r="B54" t="s">
-        <v>6</v>
+        <v>150</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F54" t="s">
-        <v>8</v>
+        <v>151</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2023,13 +2023,13 @@
         <v>6</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F55" t="s">
-        <v>61</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2037,10 +2037,7 @@
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>51</v>
-      </c>
-      <c r="C56" t="s">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>90</v>
@@ -2049,7 +2046,7 @@
         <v>121</v>
       </c>
       <c r="F56" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2063,13 +2060,13 @@
         <v>74</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F57" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2077,19 +2074,19 @@
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="C58" t="s">
         <v>74</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F58" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2097,16 +2094,19 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>78</v>
+        <v>84</v>
+      </c>
+      <c r="C59" t="s">
+        <v>74</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F59" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2114,7 +2114,7 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>65</v>
@@ -2123,7 +2123,7 @@
         <v>121</v>
       </c>
       <c r="F60" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2131,19 +2131,16 @@
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>84</v>
-      </c>
-      <c r="C61" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F61" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2151,19 +2148,19 @@
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="C62" t="s">
         <v>74</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F62" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2171,19 +2168,19 @@
         <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="C63" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F63" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2191,33 +2188,36 @@
         <v>3</v>
       </c>
       <c r="B64" t="s">
-        <v>10</v>
+        <v>92</v>
+      </c>
+      <c r="C64" t="s">
+        <v>93</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F64" t="s">
-        <v>163</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="B65" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F65" t="s">
-        <v>45</v>
+        <v>163</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2225,16 +2225,16 @@
         <v>33</v>
       </c>
       <c r="B66" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F66" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2248,10 +2248,10 @@
         <v>65</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F67" t="s">
-        <v>122</v>
+        <v>35</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2259,16 +2259,16 @@
         <v>33</v>
       </c>
       <c r="B68" t="s">
-        <v>148</v>
+        <v>34</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="F68" t="s">
-        <v>149</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2276,50 +2276,50 @@
         <v>33</v>
       </c>
       <c r="B69" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="F69" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>145</v>
+        <v>33</v>
       </c>
       <c r="B70" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F70" t="s">
-        <v>147</v>
+        <v>125</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="B71" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>64</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>152</v>
+        <v>7</v>
       </c>
       <c r="F71" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2333,10 +2333,10 @@
         <v>64</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>7</v>
+        <v>152</v>
       </c>
       <c r="F72" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2344,7 +2344,7 @@
         <v>136</v>
       </c>
       <c r="B73" t="s">
-        <v>172</v>
+        <v>137</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>64</v>
@@ -2353,41 +2353,41 @@
         <v>7</v>
       </c>
       <c r="F73" t="s">
-        <v>173</v>
+        <v>138</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="B74" t="s">
-        <v>98</v>
+        <v>172</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>152</v>
+        <v>7</v>
       </c>
       <c r="F74" t="s">
-        <v>99</v>
+        <v>173</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>9</v>
+        <v>97</v>
       </c>
       <c r="B75" t="s">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>7</v>
+        <v>152</v>
       </c>
       <c r="F75" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2395,19 +2395,16 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>59</v>
-      </c>
-      <c r="C76" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2427,7 +2424,7 @@
         <v>121</v>
       </c>
       <c r="F77" t="s">
-        <v>170</v>
+        <v>58</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2435,7 +2432,10 @@
         <v>9</v>
       </c>
       <c r="B78" t="s">
-        <v>78</v>
+        <v>59</v>
+      </c>
+      <c r="C78" t="s">
+        <v>60</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>65</v>
@@ -2444,7 +2444,7 @@
         <v>121</v>
       </c>
       <c r="F78" t="s">
-        <v>79</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2452,10 +2452,7 @@
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>6</v>
-      </c>
-      <c r="C79" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>65</v>
@@ -2464,7 +2461,7 @@
         <v>121</v>
       </c>
       <c r="F79" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -2475,7 +2472,7 @@
         <v>6</v>
       </c>
       <c r="C80" t="s">
-        <v>106</v>
+        <v>57</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>65</v>
@@ -2492,6 +2489,9 @@
         <v>9</v>
       </c>
       <c r="B81" t="s">
+        <v>6</v>
+      </c>
+      <c r="C81" t="s">
         <v>106</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -2501,7 +2501,7 @@
         <v>121</v>
       </c>
       <c r="F81" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -2512,13 +2512,13 @@
         <v>106</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F82" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -2535,7 +2535,7 @@
         <v>121</v>
       </c>
       <c r="F83" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -2546,13 +2546,13 @@
         <v>106</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F84" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -2560,7 +2560,7 @@
         <v>9</v>
       </c>
       <c r="B85" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>65</v>
@@ -2569,7 +2569,7 @@
         <v>7</v>
       </c>
       <c r="F85" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -2580,13 +2580,13 @@
         <v>131</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>121</v>
+        <v>7</v>
       </c>
       <c r="F86" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -2597,13 +2597,13 @@
         <v>131</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F87" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -2611,16 +2611,16 @@
         <v>9</v>
       </c>
       <c r="B88" t="s">
-        <v>153</v>
+        <v>131</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F88" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -2628,33 +2628,33 @@
         <v>9</v>
       </c>
       <c r="B89" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F89" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>86</v>
+        <v>9</v>
       </c>
       <c r="B90" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F90" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add motel management functionality with XML configuration and UI integration
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C18342-AD9B-4FA5-8EAA-1635730CF477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D95A554-A71F-4A5C-91A8-8353705B62A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -1737,7 +1737,7 @@
         <v>65</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F38" t="s">
         <v>29</v>
@@ -1771,7 +1771,7 @@
         <v>66</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F40" t="s">
         <v>175</v>

</xml_diff>

<commit_message>
feat: Implement commercial vehicle purchase entitlement system and update related persistence logic
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30120"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E995A0E1-4228-42CB-BA9C-DC4125537337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4426E96A-88BA-43FD-A4B7-75A96B954DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -1586,7 +1586,7 @@
         <v>64</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F27" t="s">
         <v>188</v>
@@ -1620,7 +1620,7 @@
         <v>64</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="F29" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Add control bindings and fuel management features
- Updated LSOL.ini to include control bindings for dashboard toggle, mod menu, debug menu, and interaction.
- Enhanced ControlBindings class to load control settings from LSOL.ini, with fallback to defaults for invalid or missing values.
- Introduced methods to empty and fill vehicle fuel tanks in the VehicleFuelSystem.
- Updated DebugMenuProvider to include new fuel management actions in the debug menu.
- Added unit tests for control binding overrides from LSOL.ini and for the new fuel management actions in the debug menu.
- Updated PropertyManager to handle office purchase logic, ensuring rental states are cleared when converting rentals to ownership.
- Added LSOL_files.rar to the repository.
- Updated documentation links to remove file extensions for consistency.
</commit_message>
<xml_diff>
--- a/Ideas_Fix.xlsx
+++ b/Ideas_Fix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal folders\Programmation\Games\gtav_industry_mgnt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4426E96A-88BA-43FD-A4B7-75A96B954DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBAF50E-AB11-4E05-98F3-95611AA85F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A4CB3E71-E783-455A-B26D-DD537200277B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="191">
   <si>
     <t>Context</t>
   </si>
@@ -603,6 +603,12 @@
   </si>
   <si>
     <t>Add impossible level wages</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>Notified a bug when renting a new office, the previous rent is still running</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C35E873C-977B-43F9-B6E9-42F137FEA842}">
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -2793,6 +2799,23 @@
       </c>
       <c r="F96" t="s">
         <v>187</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>30</v>
+      </c>
+      <c r="B97" t="s">
+        <v>189</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F97" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>